<commit_message>
Add Qatar University and Police College journal articles; update index and workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwpfdmnSCyeYFv2sMM8c2P
</commit_message>
<xml_diff>
--- a/مصادر_البحث.xlsx
+++ b/مصادر_البحث.xlsx
@@ -11,7 +11,7 @@
     <sheet name="ملخص" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'المصادر'!$A$1:$H$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'المصادر'!$A$1:$H$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -751,7 +751,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>الجريدة الرسمية للاتحاد L 150 في 9/6/2023 ص40–205 — لا نسخة عربية رسمية</t>
+          <t>الجريدة الرسمية للاتحاد L 150 في 9/6/2023 ص40–205 — لا نسخة عربية رسمية؛ لا يوجد مصدر بديل رسمي</t>
         </is>
       </c>
     </row>
@@ -1162,17 +1162,17 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>IMF — Qatar: Selected Issues (CR 25/48)</t>
+          <t>IMF — Qatar: 2023 Article IV Consultation, Staff Report (CR 24/43)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>صفحة ويب</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>رابط فقط</t>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>محجوب — افتحه من متصفحك</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1182,10 +1182,14 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>https://www.elibrary.imf.org/view/journals/002/2025/048/002.2025.issue-048-en.xml</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr"/>
+          <t>https://www.imf.org/-/media/files/publications/cr/2024/english/1qatea2024001.pdf</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>فبراير 2024</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1198,7 +1202,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>IMF — Staff Completes 2026 Article IV Mission to Qatar (PR 26/41)</t>
+          <t>IMF — Qatar: Selected Issues (CR 25/48)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1218,14 +1222,10 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>https://www.imf.org/en/news/articles/2026/02/11/pr26041-qatar-imf-staff-completes-2026-article-iv-mission</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>اختُتمت مشاورات 2026 في 6/5/2026؛ التقرير الكامل لم يُنشر بعد</t>
-        </is>
-      </c>
+          <t>https://www.elibrary.imf.org/view/journals/002/2025/048/002.2025.issue-048-en.xml</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1238,32 +1238,32 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>QIA — Santiago Principles Self-Assessment 2025</t>
+          <t>IMF — Staff Completes 2026 Article IV Mission to Qatar (PR 26/41)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>منزّل في المستودع</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>pdfs/04_QIA_Santiago_Self-Assessment_2025.pdf</t>
+          <t>صفحة ويب</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>رابط فقط</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>https://ifswf.org/print/pdf/node/5103</t>
+          <t>https://www.imf.org/en/news/articles/2026/02/11/pr26041-qatar-imf-staff-completes-2026-article-iv-mission</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>13 صفحة — الجهاز لا ينشر أرقامًا دقيقة لتوزيع أصوله</t>
+          <t>اختُتمت مشاورات 2026 في 6/5/2026؛ التقرير الكامل لم يُنشر بعد</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>QIA — Santiago Principles Self-Assessment 2022</t>
+          <t>QIA — Santiago Principles Self-Assessment 2025</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1293,17 +1293,17 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>pdfs/04_QIA_Santiago_Self-Assessment_2022.pdf</t>
+          <t>pdfs/04_QIA_Santiago_Self-Assessment_2025.pdf</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>https://ifswf.org/print/pdf/node/4316</t>
+          <t>https://ifswf.org/print/pdf/node/5103</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>11 صفحة</t>
+          <t>13 صفحة — الجهاز لا ينشر أرقامًا دقيقة لتوزيع أصوله</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>IFSWF — Qatar Investment Authority profile</t>
+          <t>QIA — Santiago Principles Self-Assessment 2022</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1333,15 +1333,19 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>pdfs/04_IFSWF_Qatar_QIA_Profile.pdf</t>
+          <t>pdfs/04_QIA_Santiago_Self-Assessment_2022.pdf</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>https://www.ifswf.org/sites/default/files/Qatar%20QIA_0.pdf</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr"/>
+          <t>https://ifswf.org/print/pdf/node/4316</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>11 صفحة</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1354,27 +1358,27 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>QIA — How we invest</t>
+          <t>IFSWF — Qatar Investment Authority profile</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>صفحة ويب</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>رابط فقط</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>منزّل في المستودع</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>pdfs/04_IFSWF_Qatar_QIA_Profile.pdf</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>https://www.qia.qa/en/how-we-invest/Pages/default.aspx</t>
+          <t>https://www.ifswf.org/sites/default/files/Qatar%20QIA_0.pdf</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr"/>
@@ -1385,39 +1389,35 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>السادسة — الفقه</t>
+          <t>الرابعة — الوثائق والإحصاءات</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>الماوردي، الأحكام السلطانية والولايات الدينية (مطبعة السعادة 1909)</t>
+          <t>QIA — How we invest</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>منزّل في المستودع</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>pdfs/06_الماوردي_الأحكام_السلطانية_طبعة_السعادة_1909.pdf</t>
+          <t>صفحة ويب</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>رابط فقط</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>https://archive.org/details/1327-1909</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>240 صفحة، قابلة للبحث النصي — ملك عام</t>
-        </is>
-      </c>
+          <t>https://www.qia.qa/en/how-we-invest/Pages/default.aspx</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>ابن تيمية، السياسة الشرعية في إصلاح الراعي والرعية</t>
+          <t>الماوردي، الأحكام السلطانية والولايات الدينية (مطبعة السعادة 1909)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1445,17 +1445,17 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>pdfs/06_ابن_تيمية_السياسة_الشرعية.pdf</t>
+          <t>pdfs/06_الماوردي_الأحكام_السلطانية_طبعة_السعادة_1909.pdf</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>https://archive.org/details/amatullah0911_gmail_20161011</t>
+          <t>https://archive.org/details/1327-1909</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>348 صفحة — ملك عام</t>
+          <t>240 صفحة، قابلة للبحث النصي — ملك عام</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>السنهوري، مصادر الحق في الفقه الإسلامي (ج1–3)</t>
+          <t>ابن تيمية، السياسة الشرعية في إصلاح الراعي والرعية</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1485,17 +1485,17 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>pdfs/06_السنهوري_مصادر_الحق_ج1-3.pdf</t>
+          <t>pdfs/06_ابن_تيمية_السياسة_الشرعية.pdf</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>https://archive.org/details/masadir-hak-fi-fikh-islami-senhuri</t>
+          <t>https://archive.org/details/amatullah0911_gmail_20161011</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>440 صفحة — للتحقق من الهامش 16</t>
+          <t>348 صفحة — ملك عام</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>السنهوري، مصادر الحق في الفقه الإسلامي (ج4–6)</t>
+          <t>السنهوري، مصادر الحق في الفقه الإسلامي (ج1–3)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>pdfs/06_السنهوري_مصادر_الحق_ج4-6.pdf</t>
+          <t>pdfs/06_السنهوري_مصادر_الحق_ج1-3.pdf</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>590 صفحة</t>
+          <t>440 صفحة — للتحقق من الهامش 16</t>
         </is>
       </c>
     </row>
@@ -1550,32 +1550,32 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>عبد الوهاب خلاف، السياسة الشرعية أو نظام الدولة الإسلامية</t>
+          <t>السنهوري، مصادر الحق في الفقه الإسلامي (ج4–6)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>صفحة ويب</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>رابط فقط</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>منزّل في المستودع</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>pdfs/06_السنهوري_مصادر_الحق_ج4-6.pdf</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>https://ddl.mbrf.ae/book/98418</t>
+          <t>https://archive.org/details/masadir-hak-fi-fikh-islami-senhuri</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>لا نسخة PDF حرّة — مكتبة محمد بن راشد الرقمية</t>
+          <t>590 صفحة</t>
         </is>
       </c>
     </row>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>ثروت بدوي، النظم السياسية</t>
+          <t>عبد الوهاب خلاف، السياسة الشرعية أو نظام الدولة الإسلامية</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>كتاب</t>
+          <t>صفحة ويب</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
@@ -1610,12 +1610,12 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%AB%D8%B1%D9%88%D8%AA+%D8%A8%D8%AF%D9%88%D9%8A+%D8%A7%D9%84%D9%86%D8%B8%D9%85+%D8%A7%D9%84%D8%B3%D9%8A%D8%A7%D8%B3%D9%8A%D8%A9</t>
+          <t>https://ketabonline.com/ar/books/6162</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>محمي بحقوق المؤلف — بحث في فهرس WorldCat</t>
+          <t>النص كاملًا للقراءة على الإنترنت (جامع الكتب الإسلامية) — بديل: https://ddl.mbrf.ae/book/98418</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>محمد كامل ليلة، النظم السياسية</t>
+          <t>ثروت بدوي، النظم السياسية</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D9%85%D8%AD%D9%85%D8%AF+%D9%83%D8%A7%D9%85%D9%84+%D9%84%D9%8A%D9%84%D8%A9+%D8%A7%D9%84%D9%86%D8%B8%D9%85+%D8%A7%D9%84%D8%B3%D9%8A%D8%A7%D8%B3%D9%8A%D8%A9</t>
+          <t>https://search.worldcat.org/search?q=%D8%AB%D8%B1%D9%88%D8%AA+%D8%A8%D8%AF%D9%88%D9%8A+%D8%A7%D9%84%D9%86%D8%B8%D9%85+%D8%A7%D9%84%D8%B3%D9%8A%D8%A7%D8%B3%D9%8A%D8%A9</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>السيد صبري، مبادئ القانون الدستوري</t>
+          <t>محمد كامل ليلة، النظم السياسية</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%A7%D9%84%D8%B3%D9%8A%D8%AF+%D8%B5%D8%A8%D8%B1%D9%8A+%D9%85%D8%A8%D8%A7%D8%AF%D8%A6+%D8%A7%D9%84%D9%82%D8%A7%D9%86%D9%88%D9%86+%D8%A7%D9%84%D8%AF%D8%B3%D8%AA%D9%88%D8%B1%D9%8A</t>
+          <t>https://search.worldcat.org/search?q=%D9%85%D8%AD%D9%85%D8%AF+%D9%83%D8%A7%D9%85%D9%84+%D9%84%D9%8A%D9%84%D8%A9+%D8%A7%D9%84%D9%86%D8%B8%D9%85+%D8%A7%D9%84%D8%B3%D9%8A%D8%A7%D8%B3%D9%8A%D8%A9</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>جابر جاد نصار — مؤلفاته</t>
+          <t>السيد صبري، مبادئ القانون الدستوري</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1730,7 +1730,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%AC%D8%A7%D8%A8%D8%B1+%D8%AC%D8%A7%D8%AF+%D9%86%D8%B5%D8%A7%D8%B1</t>
+          <t>https://search.worldcat.org/search?q=%D8%A7%D9%84%D8%B3%D9%8A%D8%AF+%D8%B5%D8%A8%D8%B1%D9%8A+%D9%85%D8%A8%D8%A7%D8%AF%D8%A6+%D8%A7%D9%84%D9%82%D8%A7%D9%86%D9%88%D9%86+%D8%A7%D9%84%D8%AF%D8%B3%D8%AA%D9%88%D8%B1%D9%8A</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>محمد رفعت عبد الوهاب — مؤلفاته</t>
+          <t>جابر جاد نصار — مؤلفاته</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D9%85%D8%AD%D9%85%D8%AF+%D8%B1%D9%81%D8%B9%D8%AA+%D8%B9%D8%A8%D8%AF+%D8%A7%D9%84%D9%88%D9%87%D8%A7%D8%A8</t>
+          <t>https://search.worldcat.org/search?q=%D8%AC%D8%A7%D8%A8%D8%B1+%D8%AC%D8%A7%D8%AF+%D9%86%D8%B5%D8%A7%D8%B1</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>عبد الغني بسيوني عبد الله — مؤلفاته</t>
+          <t>محمد رفعت عبد الوهاب — مؤلفاته</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%B9%D8%A8%D8%AF+%D8%A7%D9%84%D8%BA%D9%86%D9%8A+%D8%A8%D8%B3%D9%8A%D9%88%D9%86%D9%8A+%D8%B9%D8%A8%D8%AF+%D8%A7%D9%84%D9%84%D9%87</t>
+          <t>https://search.worldcat.org/search?q=%D9%85%D8%AD%D9%85%D8%AF+%D8%B1%D9%81%D8%B9%D8%AA+%D8%B9%D8%A8%D8%AF+%D8%A7%D9%84%D9%88%D9%87%D8%A7%D8%A8</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>يحيى الجمل — مؤلفاته</t>
+          <t>عبد الغني بسيوني عبد الله — مؤلفاته</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D9%8A%D8%AD%D9%8A%D9%89+%D8%A7%D9%84%D8%AC%D9%85%D9%84</t>
+          <t>https://search.worldcat.org/search?q=%D8%B9%D8%A8%D8%AF+%D8%A7%D9%84%D8%BA%D9%86%D9%8A+%D8%A8%D8%B3%D9%8A%D9%88%D9%86%D9%8A+%D8%B9%D8%A8%D8%AF+%D8%A7%D9%84%D9%84%D9%87</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>سعاد الشرقاوي — مؤلفاته</t>
+          <t>يحيى الجمل — مؤلفاته</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%B3%D8%B9%D8%A7%D8%AF+%D8%A7%D9%84%D8%B4%D8%B1%D9%82%D8%A7%D9%88%D9%8A</t>
+          <t>https://search.worldcat.org/search?q=%D9%8A%D8%AD%D9%8A%D9%89+%D8%A7%D9%84%D8%AC%D9%85%D9%84</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>حسن السيد — مؤلفاته</t>
+          <t>سعاد الشرقاوي — مؤلفاته</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%AD%D8%B3%D9%86+%D8%A7%D9%84%D8%B3%D9%8A%D8%AF</t>
+          <t>https://search.worldcat.org/search?q=%D8%B3%D8%B9%D8%A7%D8%AF+%D8%A7%D9%84%D8%B4%D8%B1%D9%82%D8%A7%D9%88%D9%8A</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>رعد ناجي الجدة — مؤلفاته</t>
+          <t>حسن السيد — مؤلفاته</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%B1%D8%B9%D8%AF+%D9%86%D8%A7%D8%AC%D9%8A+%D8%A7%D9%84%D8%AC%D8%AF%D8%A9</t>
+          <t>https://search.worldcat.org/search?q=%D8%AD%D8%B3%D9%86+%D8%A7%D9%84%D8%B3%D9%8A%D8%AF</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>سليمان محمد الطماوي — مؤلفاته</t>
+          <t>رعد ناجي الجدة — مؤلفاته</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2010,7 +2010,7 @@
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%B3%D9%84%D9%8A%D9%85%D8%A7%D9%86+%D9%85%D8%AD%D9%85%D8%AF+%D8%A7%D9%84%D8%B7%D9%85%D8%A7%D9%88%D9%8A</t>
+          <t>https://search.worldcat.org/search?q=%D8%B1%D8%B9%D8%AF+%D9%86%D8%A7%D8%AC%D9%8A+%D8%A7%D9%84%D8%AC%D8%AF%D8%A9</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>ماجد راغب الحلو — مؤلفاته</t>
+          <t>سليمان محمد الطماوي — مؤلفاته</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D9%85%D8%A7%D8%AC%D8%AF+%D8%B1%D8%A7%D8%BA%D8%A8+%D8%A7%D9%84%D8%AD%D9%84%D9%88</t>
+          <t>https://search.worldcat.org/search?q=%D8%B3%D9%84%D9%8A%D9%85%D8%A7%D9%86+%D9%85%D8%AD%D9%85%D8%AF+%D8%A7%D9%84%D8%B7%D9%85%D8%A7%D9%88%D9%8A</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>طعيمة الجرف — مؤلفاته</t>
+          <t>ماجد راغب الحلو — مؤلفاته</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%B7%D8%B9%D9%8A%D9%85%D8%A9+%D8%A7%D9%84%D8%AC%D8%B1%D9%81</t>
+          <t>https://search.worldcat.org/search?q=%D9%85%D8%A7%D8%AC%D8%AF+%D8%B1%D8%A7%D8%BA%D8%A8+%D8%A7%D9%84%D8%AD%D9%84%D9%88</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>حسن كيرة — مؤلفاته</t>
+          <t>طعيمة الجرف — مؤلفاته</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%AD%D8%B3%D9%86+%D9%83%D9%8A%D8%B1%D8%A9</t>
+          <t>https://search.worldcat.org/search?q=%D8%B7%D8%B9%D9%8A%D9%85%D8%A9+%D8%A7%D9%84%D8%AC%D8%B1%D9%81</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>عبد المنعم فرج الصدة — مؤلفاته</t>
+          <t>حسن كيرة — مؤلفاته</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%B9%D8%A8%D8%AF+%D8%A7%D9%84%D9%85%D9%86%D8%B9%D9%85+%D9%81%D8%B1%D8%AC+%D8%A7%D9%84%D8%B5%D8%AF%D8%A9</t>
+          <t>https://search.worldcat.org/search?q=%D8%AD%D8%B3%D9%86+%D9%83%D9%8A%D8%B1%D8%A9</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>علي جمال الدين عوض، عمليات البنوك من الوجهة القانونية</t>
+          <t>عبد المنعم فرج الصدة — مؤلفاته</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%B9%D9%84%D9%8A+%D8%AC%D9%85%D8%A7%D9%84+%D8%A7%D9%84%D8%AF%D9%8A%D9%86+%D8%B9%D9%88%D8%B6+%D8%B9%D9%85%D9%84%D9%8A%D8%A7%D8%AA+%D8%A7%D9%84%D8%A8%D9%86%D9%88%D9%83+%D9%85%D9%86+%D8%A7%D9%84%D9%88%D8%AC%D9%87%D8%A9+%D8%A7%D9%84%D9%82%D8%A7%D9%86%D9%88%D9%86%D9%8A%D8%A9</t>
+          <t>https://search.worldcat.org/search?q=%D8%B9%D8%A8%D8%AF+%D8%A7%D9%84%D9%85%D9%86%D8%B9%D9%85+%D9%81%D8%B1%D8%AC+%D8%A7%D9%84%D8%B5%D8%AF%D8%A9</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
@@ -2230,7 +2230,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>عادل أحمد حشيش — مؤلفاته</t>
+          <t>علي جمال الدين عوض، عمليات البنوك من الوجهة القانونية</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%B9%D8%A7%D8%AF%D9%84+%D8%A3%D8%AD%D9%85%D8%AF+%D8%AD%D8%B4%D9%8A%D8%B4</t>
+          <t>https://search.worldcat.org/search?q=%D8%B9%D9%84%D9%8A+%D8%AC%D9%85%D8%A7%D9%84+%D8%A7%D9%84%D8%AF%D9%8A%D9%86+%D8%B9%D9%88%D8%B6+%D8%B9%D9%85%D9%84%D9%8A%D8%A7%D8%AA+%D8%A7%D9%84%D8%A8%D9%86%D9%88%D9%83+%D9%85%D9%86+%D8%A7%D9%84%D9%88%D8%AC%D9%87%D8%A9+%D8%A7%D9%84%D9%82%D8%A7%D9%86%D9%88%D9%86%D9%8A%D8%A9</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>محمد ضياء الدين الريس، النظريات السياسية الإسلامية</t>
+          <t>عادل أحمد حشيش — مؤلفاته</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D9%85%D8%AD%D9%85%D8%AF+%D8%B6%D9%8A%D8%A7%D8%A1+%D8%A7%D9%84%D8%AF%D9%8A%D9%86+%D8%A7%D9%84%D8%B1%D9%8A%D8%B3+%D8%A7%D9%84%D9%86%D8%B8%D8%B1%D9%8A%D8%A7%D8%AA+%D8%A7%D9%84%D8%B3%D9%8A%D8%A7%D8%B3%D9%8A%D8%A9+%D8%A7%D9%84%D8%A5%D8%B3%D9%84%D8%A7%D9%85%D9%8A%D8%A9</t>
+          <t>https://search.worldcat.org/search?q=%D8%B9%D8%A7%D8%AF%D9%84+%D8%A3%D8%AD%D9%85%D8%AF+%D8%AD%D8%B4%D9%8A%D8%B4</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>عبد الحميد متولي، مبادئ نظام الحكم في الإسلام</t>
+          <t>محمد ضياء الدين الريس، النظريات السياسية الإسلامية</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%B9%D8%A8%D8%AF+%D8%A7%D9%84%D8%AD%D9%85%D9%8A%D8%AF+%D9%85%D8%AA%D9%88%D9%84%D9%8A+%D9%85%D8%A8%D8%A7%D8%AF%D8%A6+%D9%86%D8%B8%D8%A7%D9%85+%D8%A7%D9%84%D8%AD%D9%83%D9%85+%D9%81%D9%8A+%D8%A7%D9%84%D8%A5%D8%B3%D9%84%D8%A7%D9%85</t>
+          <t>https://search.worldcat.org/search?q=%D9%85%D8%AD%D9%85%D8%AF+%D8%B6%D9%8A%D8%A7%D8%A1+%D8%A7%D9%84%D8%AF%D9%8A%D9%86+%D8%A7%D9%84%D8%B1%D9%8A%D8%B3+%D8%A7%D9%84%D9%86%D8%B8%D8%B1%D9%8A%D8%A7%D8%AA+%D8%A7%D9%84%D8%B3%D9%8A%D8%A7%D8%B3%D9%8A%D8%A9+%D8%A7%D9%84%D8%A5%D8%B3%D9%84%D8%A7%D9%85%D9%8A%D8%A9</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>محمد سليم العوا، في النظام السياسي للدولة الإسلامية</t>
+          <t>عبد الحميد متولي، مبادئ نظام الحكم في الإسلام</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D9%85%D8%AD%D9%85%D8%AF+%D8%B3%D9%84%D9%8A%D9%85+%D8%A7%D9%84%D8%B9%D9%88%D8%A7+%D9%81%D9%8A+%D8%A7%D9%84%D9%86%D8%B8%D8%A7%D9%85+%D8%A7%D9%84%D8%B3%D9%8A%D8%A7%D8%B3%D9%8A+%D9%84%D9%84%D8%AF%D9%88%D9%84%D8%A9+%D8%A7%D9%84%D8%A5%D8%B3%D9%84%D8%A7%D9%85%D9%8A%D8%A9</t>
+          <t>https://search.worldcat.org/search?q=%D8%B9%D8%A8%D8%AF+%D8%A7%D9%84%D8%AD%D9%85%D9%8A%D8%AF+%D9%85%D8%AA%D9%88%D9%84%D9%8A+%D9%85%D8%A8%D8%A7%D8%AF%D8%A6+%D9%86%D8%B8%D8%A7%D9%85+%D8%A7%D9%84%D8%AD%D9%83%D9%85+%D9%81%D9%8A+%D8%A7%D9%84%D8%A5%D8%B3%D9%84%D8%A7%D9%85</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>توفيق الشاوي، فقه الشورى والاستشارة</t>
+          <t>محمد سليم العوا، في النظام السياسي للدولة الإسلامية</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>https://search.worldcat.org/search?q=%D8%AA%D9%88%D9%81%D9%8A%D9%82+%D8%A7%D9%84%D8%B4%D8%A7%D9%88%D9%8A+%D9%81%D9%82%D9%87+%D8%A7%D9%84%D8%B4%D9%88%D8%B1%D9%89+%D9%88%D8%A7%D9%84%D8%A7%D8%B3%D8%AA%D8%B4%D8%A7%D8%B1%D8%A9</t>
+          <t>https://search.worldcat.org/search?q=%D9%85%D8%AD%D9%85%D8%AF+%D8%B3%D9%84%D9%8A%D9%85+%D8%A7%D9%84%D8%B9%D9%88%D8%A7+%D9%81%D9%8A+%D8%A7%D9%84%D9%86%D8%B8%D8%A7%D9%85+%D8%A7%D9%84%D8%B3%D9%8A%D8%A7%D8%B3%D9%8A+%D9%84%D9%84%D8%AF%D9%88%D9%84%D8%A9+%D8%A7%D9%84%D8%A5%D8%B3%D9%84%D8%A7%D9%85%D9%8A%D8%A9</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
@@ -2425,22 +2425,22 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>السابعة — الأبحاث</t>
+          <t>السادسة — الفقه</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>«القوانين التي ترتب أحكامها صفة دستورية في التشريع القطري»، المجلة الدولية للقانون، جامعة قطر، مج10 ع2، 2021</t>
+          <t>توفيق الشاوي، فقه الشورى والاستشارة</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="E49" s="6" t="inlineStr">
-        <is>
-          <t>محجوب — افتحه من متصفحك</t>
+          <t>كتاب</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>رابط فقط</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
@@ -2450,12 +2450,12 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>https://journals.qu.edu.qa/index.php/IRL/article/download/2135/1538/2585</t>
+          <t>https://search.worldcat.org/search?q=%D8%AA%D9%88%D9%81%D9%8A%D9%82+%D8%A7%D9%84%D8%B4%D8%A7%D9%88%D9%8A+%D9%81%D9%82%D9%87+%D8%A7%D9%84%D8%B4%D9%88%D8%B1%D9%89+%D9%88%D8%A7%D9%84%D8%A7%D8%B3%D8%AA%D8%B4%D8%A7%D8%B1%D8%A9</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>خلل في شهادة TLS لخادم المجلة — تحقق من اسم الباحث</t>
+          <t>محمي بحقوق المؤلف — بحث في فهرس WorldCat</t>
         </is>
       </c>
     </row>
@@ -2470,17 +2470,17 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>«الرقابة الدستورية على الانحراف التشريعي الغائي السلبي»، المجلة الدولية للقانون، جامعة قطر</t>
+          <t>أرشيف مجلة الدراسات القانونية والأمنية — كلية الشرطة (الموقع الجديد)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="inlineStr">
-        <is>
-          <t>محجوب — افتحه من متصفحك</t>
+          <t>صفحة ويب</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>رابط فقط</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -2490,10 +2490,14 @@
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>https://journals.qu.edu.qa/index.php/IRL/article/download/4953/3112?inline=1</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr"/>
+          <t>https://jlss.moi.gov.qa/index.php/PAJ/issue/archive</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>كل الأعداد مع ملفات PDF لكل مقال</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2506,32 +2510,32 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>مجلة الدراسات القانونية والأمنية — كلية الشرطة، قطر (أرشيف الأعداد)</t>
+          <t>أناس المشيشي، «القوانين التي ترتب أحكامها صفة دستورية في التشريع القطري – محاولة لتحديد المفهوم»، المجلة الدولية للقانون (جامعة قطر)، مج10 ع2، 2021</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>صفحة ويب</t>
-        </is>
-      </c>
-      <c r="E51" s="6" t="inlineStr">
-        <is>
-          <t>محجوب — افتحه من متصفحك</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>منزّل في المستودع</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>pdfs/07_جامعة_قطر_القوانين_التي_ترتب_أحكامها_صفة_دستورية.pdf</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>https://portal.moi.gov.qa/policecollege/publications.html</t>
+          <t>https://qspace.qu.edu.qa/server/api/core/bitstreams/bef02f28-86d8-4e88-8496-400a62639158/content</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>الخادم يرفض الطلبات الآلية — اختر مقالًا من الأعداد</t>
+          <t>27 صفحة — صفحة المستودع: http://hdl.handle.net/10576/25654</t>
         </is>
       </c>
     </row>
@@ -2541,35 +2545,39 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>الثامنة — المواقع</t>
+          <t>السابعة — الأبحاث</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>مركز قطر للمال (QFC)</t>
+          <t>سارة علي الصلّابي، «الرقابة الدستورية على الانحراف التشريعي الغائي السلبي – دراسة في أحكام القضاء الدستوري في مصر ونماذج من التشريع القطري»، المجلة الدولية للقانون (جامعة قطر)، مج14 ع1، 2025</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>صفحة ويب</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="inlineStr">
-        <is>
-          <t>رابط فقط</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>منزّل في المستودع</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>pdfs/07_جامعة_قطر_الرقابة_الدستورية_على_الانحراف_التشريعي.pdf</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>https://www.qfc.qa</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="inlineStr"/>
+          <t>https://qspace.qu.edu.qa/server/api/core/bitstreams/7e52ce8e-aed5-49b8-ac18-d08a47a31f3e/content</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>28 صفحة — صفحة المستودع: http://hdl.handle.net/10576/68367</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -2577,35 +2585,39 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>الثامنة — المواقع</t>
+          <t>السابعة — الأبحاث</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>QFC — خبر إصدار إطار الأصول الرقمية 2024</t>
+          <t>امنة محمد الخاطر ومهند مختار نوح، «الدور التشريعي للسلطة التنفيذية في ظل الدستور القطري - دراسة مقارنة»، QScience Connect، مج2020 ع1، 2020</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>صفحة ويب</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="inlineStr">
-        <is>
-          <t>رابط فقط</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>منزّل في المستودع</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>pdfs/07_جامعة_قطر_الدور_التشريعي_للسلطة_التنفيذية_الدستور_القطري.pdf</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>https://www.qfc.qa/en/media-centre/news/list/qatar-financial-centre-issues-qfc-digital-assets-framework-2024</t>
-        </is>
-      </c>
-      <c r="H53" s="3" t="inlineStr"/>
+          <t>https://qspace.qu.edu.qa/server/api/core/bitstreams/21bce9b5-2181-48dc-b956-0ef7793ca0bd/content</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>16 صفحة — صفحة المستودع: http://hdl.handle.net/10576/27719</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -2613,35 +2625,39 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>الثامنة — المواقع</t>
+          <t>السابعة — الأبحاث</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>هيئة تنظيم مركز قطر للمال (QFCRA)</t>
+          <t>سونيا ملاك، «الصياغة التشريعية في القانون القطري قراءة في ضوابط صياغة النصوص القانونية»، مجلة الدراسات القانونية والأمنية، مجلد 1 عدد 1 (2021)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>صفحة ويب</t>
-        </is>
-      </c>
-      <c r="E54" s="7" t="inlineStr">
-        <is>
-          <t>رابط فقط</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>منزّل في المستودع</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>pdfs/07_مجلة_الشرطة_الصياغة_التشريعية_في_القانون_القطري.pdf</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>https://www.qfcra.com</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr"/>
+          <t>https://jlss.moi.gov.qa/index.php/PAJ/article/download/80/61</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>38 صفحة</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -2649,35 +2665,39 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>الثامنة — المواقع</t>
+          <t>السابعة — الأبحاث</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>QFCRA — استبعاد العملات المشفرة والمستقرة من إطار الأصول الرقمية</t>
+          <t>شاكر المزوغي، «خصوصية فض المنازعات الناشئة داخل أسواق الأوراق المالية في القانون القطري»، مجلة الدراسات القانونية والأمنية، مجلد 2 عدد 2 (2022)</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>صفحة ويب</t>
-        </is>
-      </c>
-      <c r="E55" s="7" t="inlineStr">
-        <is>
-          <t>رابط فقط</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>منزّل في المستودع</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>pdfs/07_مجلة_الشرطة_فض_منازعات_أسواق_الأوراق_المالية_القانون_القطري.pdf</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>https://www.qfcra.com/news/qfc-regulatory-authority-clarifies-that-cryptocurrencies-stablecoins-and-certain-other-virtual-assets-are-excluded-tokens-under-the-new-digital-assets-framework/</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="inlineStr"/>
+          <t>https://jlss.moi.gov.qa/index.php/PAJ/article/download/101/50</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>20 صفحة</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -2685,40 +2705,304 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
+          <t>السابعة — الأبحاث</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>محمد فوزي نويجي، «التنفيذ المباشر للقرارات الإدارية وتطبيقاته في القانون القطري»، مجلة الدراسات القانونية والأمنية، مجلد 2 عدد 2 (2022)</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>منزّل في المستودع</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>pdfs/07_مجلة_الشرطة_التنفيذ_المباشر_للقرارات_الإدارية.pdf</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>https://jlss.moi.gov.qa/index.php/PAJ/article/download/105/46</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>48 صفحة</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>السابعة — الأبحاث</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>حمد حامد آل مايقة الحبابي، «الاختصاص بتفسير النصوص الدستورية في القانون المقارن ومعوقاته في القانون القطري»، مجلة الدراسات القانونية والأمنية، مجلد 3 عدد 2 (2023)</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>منزّل في المستودع</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>pdfs/07_مجلة_الشرطة_تفسير_النصوص_الدستورية_القانون_القطري.pdf</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>https://jlss.moi.gov.qa/index.php/PAJ/article/download/116/36</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>48 صفحة</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>السابعة — الأبحاث</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>حسن عبد الرحيم البوهاشم السيد، «النظام القانوني للأعضاء غير المنتخبين في المجالس التشريعية الخليجية، وأثره على فاعلية أدائها»، مجلة الدراسات القانونية والأمنية، مجلد 4 عدد 1 (2024)</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>منزّل في المستودع</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>pdfs/07_مجلة_الشرطة_الأعضاء_غير_المنتخبين_المجالس_التشريعية_الخليجية.pdf</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>https://jlss.moi.gov.qa/index.php/PAJ/article/download/123/31</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>55 صفحة</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
           <t>الثامنة — المواقع</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>مركز قطر للمال (QFC)</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>صفحة ويب</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>رابط فقط</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>https://www.qfc.qa</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>الثامنة — المواقع</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>QFC — خبر إصدار إطار الأصول الرقمية 2024</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>صفحة ويب</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>رابط فقط</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>https://www.qfc.qa/en/media-centre/news/list/qatar-financial-centre-issues-qfc-digital-assets-framework-2024</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>الثامنة — المواقع</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>هيئة تنظيم مركز قطر للمال (QFCRA)</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>صفحة ويب</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>رابط فقط</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>https://www.qfcra.com</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>الثامنة — المواقع</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>QFCRA — استبعاد العملات المشفرة والمستقرة من إطار الأصول الرقمية</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>صفحة ويب</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>رابط فقط</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>https://www.qfcra.com/news/qfc-regulatory-authority-clarifies-that-cryptocurrencies-stablecoins-and-certain-other-virtual-assets-are-excluded-tokens-under-the-new-digital-assets-framework/</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>الثامنة — المواقع</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
         <is>
           <t>صندوق النقد الدولي — صفحة قطر</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>صفحة ويب</t>
         </is>
       </c>
-      <c r="E56" s="7" t="inlineStr">
+      <c r="E63" s="7" t="inlineStr">
         <is>
           <t>رابط فقط</t>
         </is>
       </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G56" s="5" t="inlineStr">
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
         <is>
           <t>https://www.imf.org/en/countries/qat</t>
         </is>
       </c>
-      <c r="H56" s="3" t="inlineStr"/>
+      <c r="H63" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H56"/>
+  <autoFilter ref="A1:H63"/>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"منزّل في المستودع,رابط فقط,محجوب — افتحه من متصفحك"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2752,21 +3036,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId47"/>
@@ -2791,12 +3075,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId89"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2841,7 +3140,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>COUNTIF('المصادر'!$E$2:$E$56,A4)</f>
+        <f>COUNTIF('المصادر'!$E$2:$E$63,A4)</f>
         <v/>
       </c>
     </row>
@@ -2852,7 +3151,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>COUNTIF('المصادر'!$E$2:$E$56,A5)</f>
+        <f>COUNTIF('المصادر'!$E$2:$E$63,A5)</f>
         <v/>
       </c>
     </row>
@@ -2863,7 +3162,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>COUNTIF('المصادر'!$E$2:$E$56,A6)</f>
+        <f>COUNTIF('المصادر'!$E$2:$E$63,A6)</f>
         <v/>
       </c>
     </row>
@@ -2897,7 +3196,7 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>COUNTIF('المصادر'!$B$2:$B$56,A10)</f>
+        <f>COUNTIF('المصادر'!$B$2:$B$63,A10)</f>
         <v/>
       </c>
     </row>
@@ -2908,7 +3207,7 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>COUNTIF('المصادر'!$B$2:$B$56,A11)</f>
+        <f>COUNTIF('المصادر'!$B$2:$B$63,A11)</f>
         <v/>
       </c>
     </row>
@@ -2919,7 +3218,7 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>COUNTIF('المصادر'!$B$2:$B$56,A12)</f>
+        <f>COUNTIF('المصادر'!$B$2:$B$63,A12)</f>
         <v/>
       </c>
     </row>
@@ -2930,7 +3229,7 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>COUNTIF('المصادر'!$B$2:$B$56,A13)</f>
+        <f>COUNTIF('المصادر'!$B$2:$B$63,A13)</f>
         <v/>
       </c>
     </row>
@@ -2941,7 +3240,7 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>COUNTIF('المصادر'!$B$2:$B$56,A14)</f>
+        <f>COUNTIF('المصادر'!$B$2:$B$63,A14)</f>
         <v/>
       </c>
     </row>
@@ -2952,7 +3251,7 @@
         </is>
       </c>
       <c r="B15" s="11">
-        <f>COUNTIF('المصادر'!$B$2:$B$56,A15)</f>
+        <f>COUNTIF('المصادر'!$B$2:$B$63,A15)</f>
         <v/>
       </c>
     </row>
@@ -2963,7 +3262,7 @@
         </is>
       </c>
       <c r="B16" s="11">
-        <f>COUNTIF('المصادر'!$B$2:$B$56,A16)</f>
+        <f>COUNTIF('المصادر'!$B$2:$B$63,A16)</f>
         <v/>
       </c>
     </row>

</xml_diff>